<commit_message>
edim-ai-blueprint: 권한·승인 정의서 v0.1
- EDIM_권한승인정의서.xlsx (6시트): 역할 4종+액션+리소스 단위 / 권한매트릭스
  (메뉴정의서 97메뉴 자동 도출, 셀 코드 ●/C/A/R/—) / 승인상태기계 13자산
  (Running Test·Test Run 선행 조건 명시) / Platform 승인 범위 8 / 문서보안등급(안)
- 산출물목록 완료 10종으로 갱신, 개요 §14·README 반영
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_산출물목록.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_산출물목록.xlsx
@@ -606,7 +606,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>34종 — 예정 20 · 완료 9 · 진행 2 · 템플릿 3</t>
+          <t>34종 — 예정 19 · 완료 10 · 진행 2 · 템플릿 3</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>① 개발 표준 정의서·권한 정의서 (P1 착수 전) ② 데이터 이행 계획서 (AI 학습과 연계, 조기 협의) ③ WBS 내용화</t>
+          <t>① 개발 표준 정의서 (P1 착수 전) ② 데이터 이행 계획서 (AI 학습과 연계, 조기 협의) ③ WBS 내용화</t>
         </is>
       </c>
     </row>
@@ -1439,24 +1439,24 @@
           <t>Excel</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>예정</t>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>v0.1</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>docs/EDIM_권한승인정의서.xlsx</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>권한 매트릭스(역할×메뉴 97)·승인 상태기계</t>
+          <t>매트릭스 97메뉴 자동 도출·승인 흐름 13·Platform 범위 8·Grade</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
edim-ai-blueprint: 개발 표준 정의서 v0.1
- 공통 원칙 6 (API-First·승인 게이트·모듈 경계·테넌트 필수·ADR)
- 명명 표준(JSON camelCase 등 프로토타입 관례 승계)·API 규약(RFC 9457·202+runId·멱등성)
- FE(React/TS·oxlint·동적 렌더러 보안)·BE(FastAPI 잠정·계층 규칙·Macro 엔진 안전)
- Git/리뷰(기능 ID 브랜치·체크리스트 5)·테스트(golden test·커버리지 80%)
- 보안·로깅(traceId·PII 금지)·CI(Jenkins 단계)·개정 트리거 5건(언어 확정 등)
- 산출물목록 완료 11종, README·개요 §14 반영
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_산출물목록.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_산출물목록.xlsx
@@ -606,7 +606,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>34종 — 예정 19 · 완료 10 · 진행 2 · 템플릿 3</t>
+          <t>34종 — 예정 18 · 완료 11 · 진행 2 · 템플릿 3</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>① 개발 표준 정의서 (P1 착수 전) ② 데이터 이행 계획서 (AI 학습과 연계, 조기 협의) ③ WBS 내용화</t>
+          <t>① 데이터 이행 계획서 (AI 학습과 연계, 조기 협의) ② WBS 내용화 ③ FVT 내용화</t>
         </is>
       </c>
     </row>
@@ -1476,27 +1476,27 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>문서</t>
-        </is>
-      </c>
-      <c r="E21" s="9" t="inlineStr">
-        <is>
-          <t>예정</t>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>v0.1</t>
         </is>
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>docs/EDIM_개발표준정의서.md</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>코딩·명명·Git·리뷰·API 규약 — P1 착수 전</t>
+          <t>언어중립 핵심+FastAPI·React/TS 기준, 개정 트리거 5건 명시</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
edim-ai-blueprint: 3차 리뷰(런타임 경로) — DB v0.4 + API 106
런타임 경로를 스키마 위에서 실행해보며 발견한 결함 9건:
- dwg_file.project_id/folder 부재 → GET /files?projectId&folder 서빙 불가 (Project Folder 규약)
- doc_control doc_no 단독 UQ → 버전 이력 행 불가 (W-11 Progress 모순) → (doc_no,version)
- 동일 대상 중복 PENDING 승인 가능 (동시성) → 부분 유니크
- sys_history 무인덱스 (이력 조회 풀스캔) / supersedure 자기참조 / pcr Type UQ /
  hierarchy 형제 이름 UQ / selection_item.resolved_slots(가격·Macro가 코드 문자열 파싱하던 결함)
- 자식 테이블 tenant_id 생략 정책 명문화 (RLS 연동)

API 95→106: Macro CRUD 5종(Studio가 저장 불가였던 치명 결함), hierarchy 검색,
비밀번호 변경, 전사 Dashboard, DRAFT Form 삭제, users/tenants 목록
회귀: FK·기능참조·규약·중복·핵심 자원 CRUD 스캔 전부 클린
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_산출물목록.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_산출물목록.xlsx
@@ -1256,7 +1256,7 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>39컴포넌트·API 95·구축 상태 반영</t>
+          <t>39컴포넌트·API 106·구축 상태 반영</t>
         </is>
       </c>
     </row>
@@ -1296,7 +1296,7 @@
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>53테이블 451컬럼 — v0.3 설계 품질 리뷰(정규화·i18n·제약) 반영</t>
+          <t>53테이블 455컬럼 — v0.4 런타임 경로 리뷰까지 반영</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
edim-ai-blueprint: 4차 검증 — DDL 실행 검증 (실 PostgreSQL 16) + INF-01 구축
- docs/ddl/edim_schema.sql: 53테이블 전체 DDL (제약·인덱스·EXCLUDE 포함) — 무오류 적용
- docs/ddl/verify_runtime.sql: 슬라이드 36 실데이터 검증 스위트
  T1 BOM 재귀 전개 — Part List Running Test 재현 (KDP 1-21-13-15 일치, 고정값·상속·손자·수량 누적)
  T2 row_key VARCHAR 결함 실증('1000'이 10:25에 포함) + row_key_num 수정 동작 증명
  T3 제약 6종 — 중복 PENDING·기간 EXCLUDE·XOR 2종·자기참조 위반 차단, doc 버전 2행 저장
  T4 Project Folder 조회 경로 동작
- 서버: postgres:16 컨테이너 추가 (~/apps/infra) → INF-01 구축완료 상태 반영
- DB 정의서 v0.4.1 (검증 이력), 산출물목록 35종(완료 12)
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_산출물목록.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_산출물목록.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="산출물목록" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'산출물목록'!$A$1:$H$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'산출물목록'!$A$1:$H$36</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -606,7 +606,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>34종 — 예정 18 · 완료 11 · 진행 2 · 템플릿 3</t>
+          <t>35종 — 예정 18 · 완료 12 · 진행 2 · 템플릿 3</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1351,32 +1351,32 @@
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>클래스 정의서</t>
+          <t>DB DDL·검증 스크립트</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>문서</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>예정</t>
+          <t>SQL</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>v0.4.1</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>docs/ddl/edim_schema.sql · verify_runtime.sql</t>
         </is>
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>도메인 모델 (개요 §14) — 백엔드 언어 확정 후</t>
+          <t>실 PG16 적용·BOM 재귀/제약 검증 통과 — 마이그레이션 도구 도입 시 초기본</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>인터페이스 정의서</t>
+          <t>클래스 정의서</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -1416,7 +1416,7 @@
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>API 상세 스펙(요청/응답/오류)·외부 연계 8종(REQ-I)</t>
+          <t>도메인 모델 (개요 §14) — 백엔드 언어 확정 후</t>
         </is>
       </c>
     </row>
@@ -1431,32 +1431,32 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>권한·승인 정의서</t>
+          <t>인터페이스 정의서</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Excel</t>
-        </is>
-      </c>
-      <c r="E20" s="12" t="inlineStr">
-        <is>
-          <t>완료</t>
+          <t>문서</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>예정</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>v0.1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
         <is>
-          <t>docs/EDIM_권한승인정의서.xlsx</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>매트릭스 97메뉴 자동 도출·승인 흐름 13·Platform 범위 8·Grade</t>
+          <t>API 상세 스펙(요청/응답/오류)·외부 연계 8종(REQ-I)</t>
         </is>
       </c>
     </row>
@@ -1471,12 +1471,12 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>개발 표준 정의서</t>
+          <t>권한·승인 정의서</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>Excel</t>
         </is>
       </c>
       <c r="E21" s="12" t="inlineStr">
@@ -1491,12 +1491,12 @@
       </c>
       <c r="G21" s="7" t="inlineStr">
         <is>
-          <t>docs/EDIM_개발표준정의서.md</t>
+          <t>docs/EDIM_권한승인정의서.xlsx</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>언어중립 핵심+FastAPI·React/TS 기준, 개정 트리거 5건 명시</t>
+          <t>매트릭스 97메뉴 자동 도출·승인 흐름 13·Platform 범위 8·Grade</t>
         </is>
       </c>
     </row>
@@ -1511,32 +1511,32 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>공통코드 정의서</t>
+          <t>개발 표준 정의서</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Excel</t>
-        </is>
-      </c>
-      <c r="E22" s="14" t="inlineStr">
-        <is>
-          <t>진행</t>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>v0.1</t>
         </is>
       </c>
       <c r="G22" s="7" t="inlineStr">
         <is>
-          <t>DB정의서 §10 포함</t>
+          <t>docs/EDIM_개발표준정의서.md</t>
         </is>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>분리 여부 협의 — 코드 16그룹</t>
+          <t>언어중립 핵심+FastAPI·React/TS 기준, 개정 트리거 5건 명시</t>
         </is>
       </c>
     </row>
@@ -1551,17 +1551,17 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>배치(Job) 정의서</t>
+          <t>공통코드 정의서</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>문서</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>예정</t>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="inlineStr">
+        <is>
+          <t>진행</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
@@ -1571,12 +1571,12 @@
       </c>
       <c r="G23" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>DB정의서 §10 포함</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>EDIM Run·AI 파이프라인·재고단가 산출 등 비동기 잡</t>
+          <t>분리 여부 협의 — 코드 16그룹</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>보고서·양식 정의서</t>
+          <t>배치(Job) 정의서</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>Print Form(견적서·PCR·작업지시서·검사성적서 등) — S-3-4</t>
+          <t>EDIM Run·AI 파이프라인·재고단가 산출 등 비동기 잡</t>
         </is>
       </c>
     </row>
@@ -1624,14 +1624,14 @@
       <c r="A25" s="5" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="15" t="inlineStr">
-        <is>
-          <t>구현·시험</t>
+      <c r="B25" s="13" t="inlineStr">
+        <is>
+          <t>설계</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>단위테스트 계획·결과</t>
+          <t>보고서·양식 정의서</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
@@ -1656,7 +1656,7 @@
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>P1 개발과 병행</t>
+          <t>Print Form(견적서·PCR·작업지시서·검사성적서 등) — S-3-4</t>
         </is>
       </c>
     </row>
@@ -1671,12 +1671,12 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>통합테스트 시나리오</t>
+          <t>단위테스트 계획·결과</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Excel</t>
+          <t>문서</t>
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr">
@@ -1696,7 +1696,7 @@
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>E2E: 코드 등록→CPQ→Run→견적 (개요 §7 워크플로우 기반)</t>
+          <t>P1 개발과 병행</t>
         </is>
       </c>
     </row>
@@ -1711,17 +1711,17 @@
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>기능확인서 (FVT)</t>
+          <t>통합테스트 시나리오</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>HTML/Excel</t>
-        </is>
-      </c>
-      <c r="E27" s="8" t="inlineStr">
-        <is>
-          <t>템플릿</t>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>예정</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
@@ -1731,12 +1731,12 @@
       </c>
       <c r="G27" s="7" t="inlineStr">
         <is>
-          <t>docs/03_기능확인서_FVT/FVT.html</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>기능정의서 178건 → 확인 항목 생성 가능</t>
+          <t>E2E: 코드 등록→CPQ→Run→견적 (개요 §7 워크플로우 기반)</t>
         </is>
       </c>
     </row>
@@ -1751,17 +1751,17 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>성능시험 계획·결과</t>
+          <t>기능확인서 (FVT)</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>문서</t>
-        </is>
-      </c>
-      <c r="E28" s="9" t="inlineStr">
-        <is>
-          <t>예정</t>
+          <t>HTML/Excel</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>템플릿</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
@@ -1771,12 +1771,12 @@
       </c>
       <c r="G28" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>docs/03_기능확인서_FVT/FVT.html</t>
         </is>
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>REQ-N-001~005 목표 검증 (산출물 1시간·BOM 30초 등)</t>
+          <t>기능정의서 178건 → 확인 항목 생성 가능</t>
         </is>
       </c>
     </row>
@@ -1791,12 +1791,12 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>결함관리대장</t>
+          <t>성능시험 계획·결과</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Excel</t>
+          <t>문서</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -1816,7 +1816,7 @@
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>시험 단계 운영</t>
+          <t>REQ-N-001~005 목표 검증 (산출물 1시간·BOM 30초 등)</t>
         </is>
       </c>
     </row>
@@ -1824,19 +1824,19 @@
       <c r="A30" s="5" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="16" t="inlineStr">
-        <is>
-          <t>이행·운영</t>
+      <c r="B30" s="15" t="inlineStr">
+        <is>
+          <t>구현·시험</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>데이터 이행 계획서</t>
+          <t>결함관리대장</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>문서</t>
+          <t>Excel</t>
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr">
@@ -1856,7 +1856,7 @@
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>★중요 — 고객 기존 도면·코드·단가·BOM 이관 + AI 학습(RAW DB) 연계</t>
+          <t>시험 단계 운영</t>
         </is>
       </c>
     </row>
@@ -1871,17 +1871,17 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>설치·배포 매뉴얼</t>
+          <t>데이터 이행 계획서</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="E31" s="14" t="inlineStr">
-        <is>
-          <t>진행</t>
+          <t>문서</t>
+        </is>
+      </c>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>예정</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
@@ -1891,12 +1891,12 @@
       </c>
       <c r="G31" s="7" t="inlineStr">
         <is>
-          <t>컴포넌트정의서 §8 구축 현황 + 서버 구축 이력</t>
+          <t>-</t>
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>Self-managed 패키지용 정식 매뉴얼 필요</t>
+          <t>★중요 — 고객 기존 도면·코드·단가·BOM 이관 + AI 학습(RAW DB) 연계</t>
         </is>
       </c>
     </row>
@@ -1911,17 +1911,17 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>운영자 매뉴얼</t>
+          <t>설치·배포 매뉴얼</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>문서</t>
-        </is>
-      </c>
-      <c r="E32" s="9" t="inlineStr">
-        <is>
-          <t>예정</t>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="E32" s="14" t="inlineStr">
+        <is>
+          <t>진행</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
@@ -1931,12 +1931,12 @@
       </c>
       <c r="G32" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>컴포넌트정의서 §8 구축 현황 + 서버 구축 이력</t>
         </is>
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>백업·모니터링·테넌트 관리·장애 대응</t>
+          <t>Self-managed 패키지용 정식 매뉴얼 필요</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>사용자 매뉴얼</t>
+          <t>운영자 매뉴얼</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
@@ -1976,7 +1976,7 @@
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>역할별(Set-up/일반/관리자) — 화면설계서 기반</t>
+          <t>백업·모니터링·테넌트 관리·장애 대응</t>
         </is>
       </c>
     </row>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>교육 계획·자료</t>
+          <t>사용자 매뉴얼</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
@@ -2016,7 +2016,7 @@
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>Set-up 사용자(코드·Macro 작성) 교육이 핵심</t>
+          <t>역할별(Set-up/일반/관리자) — 화면설계서 기반</t>
         </is>
       </c>
     </row>
@@ -2031,37 +2031,77 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
+          <t>교육 계획·자료</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>문서</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="inlineStr">
+        <is>
+          <t>예정</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G35" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
+        <is>
+          <t>Set-up 사용자(코드·Macro 작성) 교육이 핵심</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>이행·운영</t>
+        </is>
+      </c>
+      <c r="C36" s="7" t="inlineStr">
+        <is>
           <t>검수·인수 문서</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>문서</t>
         </is>
       </c>
-      <c r="E35" s="9" t="inlineStr">
+      <c r="E36" s="9" t="inlineStr">
         <is>
           <t>예정</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G35" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H35" s="7" t="inlineStr">
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G36" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H36" s="7" t="inlineStr">
         <is>
           <t>FVT 승인 연계</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H35"/>
+  <autoFilter ref="A1:H36"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
edim-ai-blueprint: 04_WBS — HTML 템플릿을 내용화된 Excel WBS로 대체
- EDIM_WBS.xlsx: SI 8단계 × P1~P5 중첩, 38 Task·44주(약 10개월) 주차 간트·담당·산출물
- 마일스톤 4 (M1 요구확정 W6 / M2 설계완료 W12 / M3 핵심 E2E 데모 W20 / M4 검수 W43)
- 시작일 2026-08-03 가정 — 스크립트 START 상수 변경 후 재생성
- WBS.html 제거, 산출물목록 완료 13종·README 갱신
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_산출물목록.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_산출물목록.xlsx
@@ -84,12 +84,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8F4FD"/>
+        <fgColor rgb="00C8E6C9"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C8E6C9"/>
+        <fgColor rgb="00E8F4FD"/>
       </patternFill>
     </fill>
     <fill>
@@ -606,7 +606,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>35종 — 예정 18 · 완료 12 · 진행 2 · 템플릿 3</t>
+          <t>35종 — 예정 18 · 완료 13 · 진행 2 · 템플릿 2</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>① 데이터 이행 계획서 (AI 학습과 연계, 조기 협의) ② WBS 내용화 ③ FVT 내용화</t>
+          <t>① 데이터 이행 계획서 (AI 학습과 연계, 조기 협의) ② FVT 내용화 ③ 인터페이스·클래스 정의서</t>
         </is>
       </c>
     </row>
@@ -836,27 +836,27 @@
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>HTML/Excel</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="inlineStr">
-        <is>
-          <t>템플릿</t>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="E5" s="11" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>v0.1</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>docs/04_WBS/WBS.html</t>
+          <t>docs/04_WBS/EDIM_WBS.xlsx</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>Phase 계획(P1~P5) 기반 내용화 필요</t>
+          <t>38 Task·44주 간트·M1~M4 — 시작일 가정, 계약 시 재산정</t>
         </is>
       </c>
     </row>
@@ -944,7 +944,7 @@
       <c r="A8" s="5" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>분석</t>
         </is>
@@ -959,7 +959,7 @@
           <t>MD</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
@@ -984,7 +984,7 @@
       <c r="A9" s="5" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>분석</t>
         </is>
@@ -999,7 +999,7 @@
           <t>Excel</t>
         </is>
       </c>
-      <c r="E9" s="12" t="inlineStr">
+      <c r="E9" s="11" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
@@ -1024,7 +1024,7 @@
       <c r="A10" s="5" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>분석</t>
         </is>
@@ -1039,7 +1039,7 @@
           <t>Excel(자동)</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
@@ -1064,7 +1064,7 @@
       <c r="A11" s="5" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>분석</t>
         </is>
@@ -1079,7 +1079,7 @@
           <t>Excel</t>
         </is>
       </c>
-      <c r="E11" s="12" t="inlineStr">
+      <c r="E11" s="11" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
@@ -1104,7 +1104,7 @@
       <c r="A12" s="5" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>분석</t>
         </is>
@@ -1119,7 +1119,7 @@
           <t>Excel</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
@@ -1144,7 +1144,7 @@
       <c r="A13" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>분석</t>
         </is>
@@ -1159,7 +1159,7 @@
           <t>MD</t>
         </is>
       </c>
-      <c r="E13" s="12" t="inlineStr">
+      <c r="E13" s="11" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
@@ -1184,7 +1184,7 @@
       <c r="A14" s="5" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>분석</t>
         </is>
@@ -1239,7 +1239,7 @@
           <t>MD+Excel</t>
         </is>
       </c>
-      <c r="E15" s="12" t="inlineStr">
+      <c r="E15" s="11" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
@@ -1279,7 +1279,7 @@
           <t>MD+Excel</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
@@ -1319,7 +1319,7 @@
           <t>HTML</t>
         </is>
       </c>
-      <c r="E17" s="12" t="inlineStr">
+      <c r="E17" s="11" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
@@ -1359,7 +1359,7 @@
           <t>SQL</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
@@ -1479,7 +1479,7 @@
           <t>Excel</t>
         </is>
       </c>
-      <c r="E21" s="12" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>완료</t>
         </is>
@@ -1519,7 +1519,7 @@
           <t>MD</t>
         </is>
       </c>
-      <c r="E22" s="12" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>완료</t>
         </is>

</xml_diff>

<commit_message>
edim-ai-blueprint: 인터페이스 정의서 v0.1 + OpenAPI 3.1 자동 생성 체계
- docs/api/edim-openapi.yaml: 컴포넌트 APIS 목록에서 자동 생성 (93경로·105오퍼레이션·
  52스키마) — openapi-spec-validator 검증 통과, 단일 소스 동기 보장
- EDIM_인터페이스정의서.md: 공통 규약(JWT·Problem 오류 카탈로그·커서·202+runId·멱등),
  BOM 전개 시나리오(verify_runtime T1과 동일 구조), 서비스별 총괄 16, WS 채널,
  외부 연계 8종 상세(어댑터 공통 원칙: 재시도 큐·아웃박스), 변경 관리 규칙
- 산출물목록 완료 16종, README 갱신
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_산출물목록.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_산출물목록.xlsx
@@ -598,7 +598,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>35종 — 예정 18 · 완료 15 · 진행 2</t>
+          <t>35종 — 예정 17 · 완료 16 · 진행 2</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>① 인터페이스 정의서 (OpenAPI) ② 클래스 정의서 ③ 착수 문서(수행계획·위험대장·보안계획)</t>
+          <t>① 클래스 정의서 ② 착수 문서(수행계획·위험대장·보안계획) ③ 배치·보고서양식 정의서</t>
         </is>
       </c>
     </row>
@@ -1524,17 +1524,17 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>문서</t>
-        </is>
-      </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>예정</t>
+          <t>MD+YAML</t>
+        </is>
+      </c>
+      <c r="E20" s="10" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>v0.1</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
@@ -1544,12 +1544,12 @@
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>docs/EDIM_인터페이스정의서.md · docs/api/edim-openapi.yaml</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>API 상세 스펙(요청/응답/오류)·외부 연계 8종(REQ-I)</t>
+          <t>OpenAPI 3.1 자동 생성(105 op·52 스키마)+외부 연계 8종</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
edim-ai-blueprint: 디자인 시안 B (Dense Enterprise) — 레거시 문법 조사·적용
- 조사(B-01): SAP GUI(조회밴드·F8 리듬)·더존/영림원(MDI·F-key·노란 필수셀·그리드 문법)·
  AutoCAD(커맨드라인·좌표 상태바)·Excel(활성 셀·인라인 편집) — 채택 근거 표
- 토큰(B-02): 본문 11.5px·컨트롤 22px·그리드 24px·radius 0-2·선이 그림자 대체 (행밀도 +70%)
- 화면: B-03 CPQ(MDI 탭·조회밴드·커맨드라인·그리드 스택·F-key 상태바),
  B-04 코드 등록(마스터-디테일·노란 필수/대기), B-05 Run(단계·산출물 2그리드+다음행동 열)
- B-06 권고: 하이브리드 — 업무 화면(~85메뉴)=B안, 브랜드 접점(로그인·Dashboard·모바일)=A안
- A↔B 상호 링크, 산출물 37종(완료 19)
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/EDIM_산출물목록.xlsx
+++ b/edim-ai-blueprint/docs/EDIM_산출물목록.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="산출물목록" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'산출물목록'!$A$1:$H$37</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'산출물목록'!$A$1:$H$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -598,7 +598,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>36종 — 예정 16 · 완료 18 · 진행 2</t>
+          <t>37종 — 예정 16 · 완료 19 · 진행 2</t>
         </is>
       </c>
     </row>
@@ -637,7 +637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1474,7 +1474,7 @@
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>디자인 시안 (Hi-Fi)</t>
+          <t>디자인 시안 A (Modern)</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -1499,12 +1499,12 @@
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>docs/EDIM_디자인시안.html · https://edim.seekerslab.com/design/hifi/</t>
+          <t>docs/EDIM_디자인시안.html · /design/hifi/</t>
         </is>
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>디자인 시스템(토큰)+핵심 6페이지 — 개발 시 CSS 변수 이식</t>
+          <t>브랜드 접점용(로그인·Dashboard·모바일) — B-06 권고 참조</t>
         </is>
       </c>
     </row>
@@ -1519,12 +1519,12 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>클래스 정의서</t>
+          <t>디자인 시안 B (Dense) ★권고</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>HTML</t>
         </is>
       </c>
       <c r="E20" s="10" t="inlineStr">
@@ -1544,12 +1544,12 @@
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>docs/EDIM_클래스정의서.md</t>
+          <t>docs/EDIM_디자인시안_B_dense.html · /design/dense/</t>
         </is>
       </c>
       <c r="I20" s="7" t="inlineStr">
         <is>
-          <t>언어 중립 — 11도메인·Aggregate 22·인바리언트↔DB제약 대응표</t>
+          <t>레거시 패턴 조사(SAP·더존·CAD·Excel)+22px 컨트롤+MDI·F-key — 업무 화면 표준</t>
         </is>
       </c>
     </row>
@@ -1564,12 +1564,12 @@
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>인터페이스 정의서</t>
+          <t>클래스 정의서</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>MD+YAML</t>
+          <t>MD</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
@@ -1589,12 +1589,12 @@
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>docs/EDIM_인터페이스정의서.md · docs/api/edim-openapi.yaml</t>
+          <t>docs/EDIM_클래스정의서.md</t>
         </is>
       </c>
       <c r="I21" s="7" t="inlineStr">
         <is>
-          <t>OpenAPI 3.1 자동 생성(105 op·52 스키마)+외부 연계 8종</t>
+          <t>언어 중립 — 11도메인·Aggregate 22·인바리언트↔DB제약 대응표</t>
         </is>
       </c>
     </row>
@@ -1609,12 +1609,12 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>권한·승인 정의서</t>
+          <t>인터페이스 정의서</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Excel</t>
+          <t>MD+YAML</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
@@ -1634,12 +1634,12 @@
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>docs/EDIM_권한승인정의서.xlsx</t>
+          <t>docs/EDIM_인터페이스정의서.md · docs/api/edim-openapi.yaml</t>
         </is>
       </c>
       <c r="I22" s="7" t="inlineStr">
         <is>
-          <t>매트릭스 97메뉴 자동 도출·승인 흐름 13·Platform 범위 8·Grade</t>
+          <t>OpenAPI 3.1 자동 생성(105 op·52 스키마)+외부 연계 8종</t>
         </is>
       </c>
     </row>
@@ -1654,12 +1654,12 @@
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>개발 표준 정의서</t>
+          <t>권한·승인 정의서</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>MD</t>
+          <t>Excel</t>
         </is>
       </c>
       <c r="E23" s="10" t="inlineStr">
@@ -1679,12 +1679,12 @@
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>docs/EDIM_개발표준정의서.md</t>
+          <t>docs/EDIM_권한승인정의서.xlsx</t>
         </is>
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>언어중립 핵심+FastAPI·React/TS 기준, 개정 트리거 5건 명시</t>
+          <t>매트릭스 97메뉴 자동 도출·승인 흐름 13·Platform 범위 8·Grade</t>
         </is>
       </c>
     </row>
@@ -1699,22 +1699,22 @@
       </c>
       <c r="C24" s="7" t="inlineStr">
         <is>
-          <t>공통코드 정의서</t>
+          <t>개발 표준 정의서</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Excel</t>
-        </is>
-      </c>
-      <c r="E24" s="13" t="inlineStr">
-        <is>
-          <t>진행</t>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="E24" s="10" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>v0.1</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -1724,12 +1724,12 @@
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>DB정의서 §10 포함</t>
+          <t>docs/EDIM_개발표준정의서.md</t>
         </is>
       </c>
       <c r="I24" s="7" t="inlineStr">
         <is>
-          <t>분리 여부 협의 — 코드 16그룹</t>
+          <t>언어중립 핵심+FastAPI·React/TS 기준, 개정 트리거 5건 명시</t>
         </is>
       </c>
     </row>
@@ -1744,17 +1744,17 @@
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>배치(Job) 정의서</t>
+          <t>공통코드 정의서</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>문서</t>
-        </is>
-      </c>
-      <c r="E25" s="8" t="inlineStr">
-        <is>
-          <t>예정</t>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>진행</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
@@ -1769,12 +1769,12 @@
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>DB정의서 §10 포함</t>
         </is>
       </c>
       <c r="I25" s="7" t="inlineStr">
         <is>
-          <t>EDIM Run·AI 파이프라인·재고단가 산출 등 비동기 잡</t>
+          <t>분리 여부 협의 — 코드 16그룹</t>
         </is>
       </c>
     </row>
@@ -1789,7 +1789,7 @@
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>보고서·양식 정의서</t>
+          <t>배치(Job) 정의서</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -1819,7 +1819,7 @@
       </c>
       <c r="I26" s="7" t="inlineStr">
         <is>
-          <t>Print Form(견적서·PCR·작업지시서·검사성적서 등) — S-3-4</t>
+          <t>EDIM Run·AI 파이프라인·재고단가 산출 등 비동기 잡</t>
         </is>
       </c>
     </row>
@@ -1827,14 +1827,14 @@
       <c r="A27" s="5" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="14" t="inlineStr">
-        <is>
-          <t>구현·시험</t>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>설계</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>단위테스트 계획·결과</t>
+          <t>보고서·양식 정의서</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>P1 개발과 병행</t>
+          <t>Print Form(견적서·PCR·작업지시서·검사성적서 등) — S-3-4</t>
         </is>
       </c>
     </row>
@@ -1879,12 +1879,12 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>통합테스트 시나리오</t>
+          <t>단위테스트 계획·결과</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>Excel</t>
+          <t>문서</t>
         </is>
       </c>
       <c r="E28" s="8" t="inlineStr">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="I28" s="7" t="inlineStr">
         <is>
-          <t>E2E: 코드 등록→CPQ→Run→견적 (개요 §7 워크플로우 기반)</t>
+          <t>P1 개발과 병행</t>
         </is>
       </c>
     </row>
@@ -1924,22 +1924,22 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>기능확인서 (FVT)</t>
+          <t>통합테스트 시나리오</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Excel(자동)</t>
-        </is>
-      </c>
-      <c r="E29" s="10" t="inlineStr">
-        <is>
-          <t>완료</t>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>예정</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>v0.1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
@@ -1949,12 +1949,12 @@
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>docs/03_기능확인서_FVT/EDIM_기능확인서.xlsx</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I29" s="7" t="inlineStr">
         <is>
-          <t>기능 178·비기능 22 자동 생성 — 판정 기입 후 버전 고정</t>
+          <t>E2E: 코드 등록→CPQ→Run→견적 (개요 §7 워크플로우 기반)</t>
         </is>
       </c>
     </row>
@@ -1969,22 +1969,22 @@
       </c>
       <c r="C30" s="7" t="inlineStr">
         <is>
-          <t>성능시험 계획·결과</t>
+          <t>기능확인서 (FVT)</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>문서</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>예정</t>
+          <t>Excel(자동)</t>
+        </is>
+      </c>
+      <c r="E30" s="10" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>v0.1</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
@@ -1994,12 +1994,12 @@
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>docs/03_기능확인서_FVT/EDIM_기능확인서.xlsx</t>
         </is>
       </c>
       <c r="I30" s="7" t="inlineStr">
         <is>
-          <t>REQ-N-001~005 목표 검증 (산출물 1시간·BOM 30초 등)</t>
+          <t>기능 178·비기능 22 자동 생성 — 판정 기입 후 버전 고정</t>
         </is>
       </c>
     </row>
@@ -2014,12 +2014,12 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>결함관리대장</t>
+          <t>성능시험 계획·결과</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Excel</t>
+          <t>문서</t>
         </is>
       </c>
       <c r="E31" s="8" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="I31" s="7" t="inlineStr">
         <is>
-          <t>시험 단계 운영</t>
+          <t>REQ-N-001~005 목표 검증 (산출물 1시간·BOM 30초 등)</t>
         </is>
       </c>
     </row>
@@ -2052,29 +2052,29 @@
       <c r="A32" s="5" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="15" t="inlineStr">
-        <is>
-          <t>이행·운영</t>
+      <c r="B32" s="14" t="inlineStr">
+        <is>
+          <t>구현·시험</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>데이터 이행 계획서</t>
+          <t>결함관리대장</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>MD</t>
-        </is>
-      </c>
-      <c r="E32" s="10" t="inlineStr">
-        <is>
-          <t>완료</t>
+          <t>Excel</t>
+        </is>
+      </c>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>예정</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>v0.1</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
@@ -2084,12 +2084,12 @@
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>docs/EDIM_데이터이행계획서.md</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I32" s="7" t="inlineStr">
         <is>
-          <t>9대상·5단계·검증 6기준 — 조사(2.3) 후 v0.2 갱신</t>
+          <t>시험 단계 운영</t>
         </is>
       </c>
     </row>
@@ -2104,7 +2104,7 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>설치·배포 매뉴얼</t>
+          <t>데이터 이행 계획서</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
@@ -2112,14 +2112,14 @@
           <t>MD</t>
         </is>
       </c>
-      <c r="E33" s="13" t="inlineStr">
-        <is>
-          <t>진행</t>
+      <c r="E33" s="10" t="inlineStr">
+        <is>
+          <t>완료</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>v0.1</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
@@ -2129,12 +2129,12 @@
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>컴포넌트정의서 §8 구축 현황 + 서버 구축 이력</t>
+          <t>docs/EDIM_데이터이행계획서.md</t>
         </is>
       </c>
       <c r="I33" s="7" t="inlineStr">
         <is>
-          <t>Self-managed 패키지용 정식 매뉴얼 필요</t>
+          <t>9대상·5단계·검증 6기준 — 조사(2.3) 후 v0.2 갱신</t>
         </is>
       </c>
     </row>
@@ -2149,17 +2149,17 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>운영자 매뉴얼</t>
+          <t>설치·배포 매뉴얼</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>문서</t>
-        </is>
-      </c>
-      <c r="E34" s="8" t="inlineStr">
-        <is>
-          <t>예정</t>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="E34" s="13" t="inlineStr">
+        <is>
+          <t>진행</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
@@ -2174,12 +2174,12 @@
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>컴포넌트정의서 §8 구축 현황 + 서버 구축 이력</t>
         </is>
       </c>
       <c r="I34" s="7" t="inlineStr">
         <is>
-          <t>백업·모니터링·테넌트 관리·장애 대응</t>
+          <t>Self-managed 패키지용 정식 매뉴얼 필요</t>
         </is>
       </c>
     </row>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>사용자 매뉴얼</t>
+          <t>운영자 매뉴얼</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
@@ -2224,7 +2224,7 @@
       </c>
       <c r="I35" s="7" t="inlineStr">
         <is>
-          <t>역할별(Set-up/일반/관리자) — 화면설계서 기반</t>
+          <t>백업·모니터링·테넌트 관리·장애 대응</t>
         </is>
       </c>
     </row>
@@ -2239,7 +2239,7 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>교육 계획·자료</t>
+          <t>사용자 매뉴얼</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="I36" s="7" t="inlineStr">
         <is>
-          <t>Set-up 사용자(코드·Macro 작성) 교육이 핵심</t>
+          <t>역할별(Set-up/일반/관리자) — 화면설계서 기반</t>
         </is>
       </c>
     </row>
@@ -2284,42 +2284,87 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
+          <t>교육 계획·자료</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>문서</t>
+        </is>
+      </c>
+      <c r="E37" s="8" t="inlineStr">
+        <is>
+          <t>예정</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I37" s="7" t="inlineStr">
+        <is>
+          <t>Set-up 사용자(코드·Macro 작성) 교육이 핵심</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="15" t="inlineStr">
+        <is>
+          <t>이행·운영</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
           <t>검수·인수 문서</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
+      <c r="D38" s="5" t="inlineStr">
         <is>
           <t>문서</t>
         </is>
       </c>
-      <c r="E37" s="8" t="inlineStr">
+      <c r="E38" s="8" t="inlineStr">
         <is>
           <t>예정</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G37" s="5" t="inlineStr">
-        <is>
-          <t>미정</t>
-        </is>
-      </c>
-      <c r="H37" s="7" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I37" s="7" t="inlineStr">
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="inlineStr">
+        <is>
+          <t>미정</t>
+        </is>
+      </c>
+      <c r="H38" s="7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I38" s="7" t="inlineStr">
         <is>
           <t>FVT 승인 연계</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H37"/>
+  <autoFilter ref="A1:H38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>